<commit_message>
Add Python class examples and exercises for modules 1-4
Added multiple Python scripts covering conditional statements, logical operators, loops, functions, and a simple ATM simulation for class exercises. Also included example spreadsheet and document files for logical operators and loops. These resources support foundational programming concepts for students.
</commit_message>
<xml_diff>
--- a/PythonIA/Módulo 1 Fundamentos Modernos de programación con Python/Clase2/Operadores_Logicos.xlsx
+++ b/PythonIA/Módulo 1 Fundamentos Modernos de programación con Python/Clase2/Operadores_Logicos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f109f360a9574d0/Documentos/Projects/DevSeniorCode/Clase2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f109f360a9574d0/Documentos/GitHub/DevseniorCode/PythonSeniorAI/PythonIA/Módulo 1 Fundamentos Modernos de programación con Python/Clase2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{57BEB133-4D45-45C2-B474-00363B5AB44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6965F57-C6E0-45BD-BBB8-815ED9E9C3DF}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{57BEB133-4D45-45C2-B474-00363B5AB44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{804623AB-7604-4D72-9222-59042566BE39}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7360" xr2:uid="{24008A49-332E-4BD7-9228-5BAA2DB27E51}"/>
+    <workbookView minimized="1" xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7360" xr2:uid="{24008A49-332E-4BD7-9228-5BAA2DB27E51}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -483,6 +483,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3562956D-9E92-4B6E-A9DC-418AD2E0FF87}">
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="7" max="7" width="15.26953125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>